<commit_message>
update startServer, bug tracker update
</commit_message>
<xml_diff>
--- a/bug-tracker/UBA-bugs-tracker.xlsx
+++ b/bug-tracker/UBA-bugs-tracker.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amicell\uba6-work\UBA6-release\bug-tracker\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\AnalysisResults\UBA-6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCF7DE11-6EAA-40AD-A69A-9867511624B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C810DBB-6CF4-4B42-B641-328815DD2831}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5B816FF3-3B79-4319-AB68-882518EDFCB6}"/>
   </bookViews>
@@ -34,11 +34,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="76">
   <si>
     <t>Num</t>
   </si>
   <si>
+    <t>Date</t>
+  </si>
+  <si>
     <t>Bug</t>
   </si>
   <si>
@@ -111,6 +114,9 @@
     <t>26.07.2026</t>
   </si>
   <si>
+    <t>Natasha</t>
+  </si>
+  <si>
     <t>כאשר משנים תוכנית טעינה/ פריקה ועושים Save and Run התוכנה לא נותנת להפעלה מפעם הראשונה.</t>
   </si>
   <si>
@@ -189,53 +195,81 @@
     <t>זרם טעינה, ללא מתן הנחיית טעינה</t>
   </si>
   <si>
+    <t>זרם טעינה- סטייה</t>
+  </si>
+  <si>
+    <t>בהגדת זרם טעינה 50mA בפועל הזרם שמכשיר רושם על הצג  ובגרף 42mA. בהגדרת זרם טעינה 30mA בפועל  נצפה זרם טעינה 24mA.</t>
+  </si>
+  <si>
+    <t>29.07.2026</t>
+  </si>
+  <si>
+    <t>checked in new version (28/7)</t>
+  </si>
+  <si>
+    <t>new feature in version (28/7)</t>
+  </si>
+  <si>
+    <t>neet to consult with Tomer</t>
+  </si>
+  <si>
+    <t>dc 4.8 v cuff off, then charge</t>
+  </si>
+  <si>
+    <t>inside test definition</t>
+  </si>
+  <si>
+    <t>טעינה - DUAL</t>
+  </si>
+  <si>
+    <t>זרם טעינה שהוגדר 400 מיליאמפר, כאשר בפועל הטעינה בוצעה ב 12-19 מיליאמפר</t>
+  </si>
+  <si>
+    <t>higth</t>
+  </si>
+  <si>
+    <t>DUAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">בלחיצה על STOP במכשיר עצמו : בWEB התוכנית הסתיימה ללא התרעה על הסיום וללא אופציה לשמירת נתונים, כאשר בפועל המכשיר המשיך לפרוק את הסוללה. </t>
+  </si>
+  <si>
+    <t>29.07.2027</t>
+  </si>
+  <si>
+    <t>Status Date</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
     <t>Approved by</t>
   </si>
   <si>
     <t>Approve Date</t>
   </si>
   <si>
-    <t>Open Date</t>
-  </si>
-  <si>
-    <t>Status Date</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>checked in new version (28/7)</t>
-  </si>
-  <si>
-    <t>new feature in version (28/7)</t>
-  </si>
-  <si>
-    <t>זרם טעינה- סטייה</t>
-  </si>
-  <si>
-    <t>בהגדת זרם טעינה 50mA בפועל הזרם שמכשיר רושם על הצג  ובגרף 42mA. בהגדרת זרם טעינה 30mA בפועל  נצפה זרם טעינה 24mA.</t>
-  </si>
-  <si>
-    <t>29.07.2026</t>
-  </si>
-  <si>
     <t>Note</t>
   </si>
   <si>
-    <t>neet to consult with Tomer</t>
-  </si>
-  <si>
-    <t>dc 4.8 v cuff off, then charge</t>
-  </si>
-  <si>
-    <t>inside test definition</t>
+    <t>FAIL</t>
+  </si>
+  <si>
+    <t>נדרש להוסיף אופציה לסינון/בחירה למחיקה
+לאחר מחיקה של 3 שורות מתוצאות המערכת נתקעת ולא ניתנת לתפעול, רק כיבוי והדלקה מחדש</t>
+  </si>
+  <si>
+    <t xml:space="preserve">לאחר עדכון גרסה כל התוכניות שנבנו נמחקו, כמו כן גם התוצאות שנשמרו נמחקו. </t>
+  </si>
+  <si>
+    <t>עדכון גרסה</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -272,6 +306,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -299,7 +340,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -313,10 +354,10 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -324,6 +365,12 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -639,58 +686,57 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E8ABA1E-CC26-499E-82DE-E3065ED1E830}">
-  <dimension ref="A3:L22"/>
+  <dimension ref="A3:L47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
     <col min="2" max="2" width="42.5703125" customWidth="1"/>
-    <col min="3" max="3" width="76.140625" customWidth="1"/>
-    <col min="4" max="4" width="15.7109375" customWidth="1"/>
-    <col min="5" max="5" width="11.28515625" customWidth="1"/>
-    <col min="6" max="6" width="11.42578125" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" customWidth="1"/>
-    <col min="8" max="8" width="13.5703125" customWidth="1"/>
-    <col min="9" max="9" width="28.7109375" customWidth="1"/>
-    <col min="10" max="10" width="16.140625" customWidth="1"/>
-    <col min="11" max="11" width="12.85546875" customWidth="1"/>
+    <col min="3" max="3" width="72.85546875" customWidth="1"/>
+    <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.85546875" customWidth="1"/>
+    <col min="8" max="8" width="11" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="28" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="34.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>53</v>
-      </c>
       <c r="E3" s="4" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="L3" s="4" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -698,22 +744,28 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="5">
+        <v>8</v>
+      </c>
+      <c r="D4" s="6">
         <v>45116</v>
       </c>
-      <c r="E4" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>9</v>
+      <c r="E4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -721,22 +773,22 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="6">
+        <v>45116</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G5" s="7" t="s">
         <v>11</v>
-      </c>
-      <c r="C5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="5">
-        <v>45116</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
@@ -744,22 +796,22 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D6" s="5">
+        <v>15</v>
+      </c>
+      <c r="D6" s="6">
         <v>45116</v>
       </c>
-      <c r="E6" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>9</v>
+      <c r="E6" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
@@ -767,22 +819,22 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7" s="5">
+        <v>17</v>
+      </c>
+      <c r="D7" s="6">
         <v>45116</v>
       </c>
-      <c r="E7" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>9</v>
+      <c r="E7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
@@ -790,22 +842,28 @@
         <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8" s="5">
+        <v>20</v>
+      </c>
+      <c r="D8" s="6">
         <v>45116</v>
       </c>
-      <c r="E8" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>9</v>
+      <c r="E8" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
@@ -813,22 +871,22 @@
         <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C9" t="s">
-        <v>21</v>
-      </c>
-      <c r="D9" s="5">
+        <v>22</v>
+      </c>
+      <c r="D9" s="6">
         <v>45116</v>
       </c>
-      <c r="E9" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>9</v>
+      <c r="E9" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
@@ -836,56 +894,58 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" t="s">
         <v>23</v>
       </c>
-      <c r="C10" t="s">
-        <v>22</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>9</v>
+      <c r="D10" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="I10" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I10" s="5" t="s">
         <v>56</v>
       </c>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
     </row>
     <row r="11" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D11" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="E11" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>9</v>
+      <c r="D11" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="H11" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="I11" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I11" s="5" t="s">
         <v>56</v>
       </c>
     </row>
@@ -894,27 +954,27 @@
         <v>9</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C12" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="H12" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="G12" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="I12" s="6" t="s">
+      <c r="I12" s="5" t="s">
         <v>56</v>
       </c>
     </row>
@@ -923,51 +983,60 @@
         <v>10</v>
       </c>
       <c r="B13" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C13" t="s">
-        <v>35</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F13" s="6" t="s">
-        <v>9</v>
+        <v>37</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>11</v>
       </c>
-      <c r="B14" t="s">
-        <v>32</v>
+      <c r="B14" s="10" t="s">
+        <v>34</v>
       </c>
       <c r="C14" t="s">
-        <v>33</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="G14" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="H14" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="I14" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I14" s="5" t="s">
         <v>57</v>
+      </c>
+      <c r="J14" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K14" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
@@ -975,22 +1044,22 @@
         <v>12</v>
       </c>
       <c r="B15" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C15" t="s">
-        <v>38</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>9</v>
+        <v>40</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="30" x14ac:dyDescent="0.25">
@@ -998,22 +1067,22 @@
         <v>13</v>
       </c>
       <c r="B16" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>9</v>
+        <v>42</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -1021,25 +1090,25 @@
         <v>14</v>
       </c>
       <c r="B17" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F17" s="6" t="s">
-        <v>9</v>
+        <v>44</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="I17" s="6" t="s">
-        <v>62</v>
+        <v>18</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -1047,25 +1116,25 @@
         <v>15</v>
       </c>
       <c r="B18" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C18" t="s">
-        <v>44</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="E18" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F18" s="6" t="s">
-        <v>9</v>
+        <v>46</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="I18" s="6" t="s">
-        <v>63</v>
+        <v>18</v>
+      </c>
+      <c r="I18" s="5" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -1073,25 +1142,25 @@
         <v>16</v>
       </c>
       <c r="B19" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="E19" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F19" s="6" t="s">
-        <v>9</v>
+        <v>48</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="I19" s="6" t="s">
-        <v>64</v>
+        <v>18</v>
+      </c>
+      <c r="I19" s="5" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -1099,22 +1168,22 @@
         <v>17</v>
       </c>
       <c r="B20" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C20" t="s">
-        <v>48</v>
-      </c>
-      <c r="D20" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="E20" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F20" s="6" t="s">
-        <v>9</v>
+        <v>50</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -1122,25 +1191,25 @@
         <v>18</v>
       </c>
       <c r="B21" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="D21" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="E21" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F21" s="6" t="s">
-        <v>9</v>
+        <v>51</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="I21" s="6" t="s">
-        <v>62</v>
+        <v>18</v>
+      </c>
+      <c r="I21" s="5" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -1148,23 +1217,158 @@
         <v>19</v>
       </c>
       <c r="B22" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D22" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="E22" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F22" s="6" t="s">
-        <v>9</v>
+        <v>54</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>17</v>
-      </c>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="1">
+        <v>20</v>
+      </c>
+      <c r="B23" t="s">
+        <v>61</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G23" s="8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A24" s="1">
+        <v>21</v>
+      </c>
+      <c r="B24" t="s">
+        <v>64</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G24" s="8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
+        <v>22</v>
+      </c>
+      <c r="B25" t="s">
+        <v>75</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G25" s="8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C26" s="2"/>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C27" s="2"/>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C28" s="2"/>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C29" s="2"/>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C30" s="2"/>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C31" s="2"/>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C32" s="2"/>
+    </row>
+    <row r="33" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C33" s="2"/>
+    </row>
+    <row r="34" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C34" s="2"/>
+    </row>
+    <row r="35" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C35" s="2"/>
+    </row>
+    <row r="36" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C36" s="2"/>
+    </row>
+    <row r="37" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C37" s="2"/>
+    </row>
+    <row r="38" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C38" s="2"/>
+    </row>
+    <row r="39" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C39" s="2"/>
+    </row>
+    <row r="40" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C40" s="2"/>
+    </row>
+    <row r="41" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C41" s="2"/>
+    </row>
+    <row r="42" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C42" s="2"/>
+    </row>
+    <row r="43" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C43" s="2"/>
+    </row>
+    <row r="44" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C44" s="2"/>
+    </row>
+    <row r="45" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C45" s="2"/>
+    </row>
+    <row r="46" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C46" s="2"/>
+    </row>
+    <row r="47" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C47" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
update SW version - Jul 30th
</commit_message>
<xml_diff>
--- a/bug-tracker/UBA-bugs-tracker.xlsx
+++ b/bug-tracker/UBA-bugs-tracker.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\AnalysisResults\UBA-6\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\DEV\UBA6-release\bug-tracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C810DBB-6CF4-4B42-B641-328815DD2831}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1BD46042-F4AD-4D5A-9F5C-6ABB85830967}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5B816FF3-3B79-4319-AB68-882518EDFCB6}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{5B816FF3-3B79-4319-AB68-882518EDFCB6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="79">
   <si>
     <t>Num</t>
   </si>
@@ -263,6 +264,15 @@
   </si>
   <si>
     <t>עדכון גרסה</t>
+  </si>
+  <si>
+    <t>30.07.2026</t>
+  </si>
+  <si>
+    <t>checked in ver Jul 30th</t>
+  </si>
+  <si>
+    <t>checked in ver Jul 30th, see also bug #12</t>
   </si>
 </sst>
 </file>
@@ -340,7 +350,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -372,6 +382,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -390,9 +406,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -430,7 +446,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -536,7 +552,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -678,7 +694,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -687,21 +703,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E8ABA1E-CC26-499E-82DE-E3065ED1E830}">
   <dimension ref="A3:L47"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="1"/>
-    <col min="2" max="2" width="42.5703125" customWidth="1"/>
-    <col min="3" max="3" width="72.85546875" customWidth="1"/>
-    <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.85546875" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" style="1"/>
+    <col min="2" max="2" width="42.5546875" customWidth="1"/>
+    <col min="3" max="3" width="72.88671875" customWidth="1"/>
+    <col min="4" max="4" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.88671875" customWidth="1"/>
     <col min="8" max="8" width="11" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="28" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="34.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="37.44140625" customWidth="1"/>
+    <col min="10" max="10" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="34.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>0</v>
       </c>
@@ -739,7 +755,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>1</v>
       </c>
@@ -768,7 +784,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>2</v>
       </c>
@@ -790,8 +806,9 @@
       <c r="G5" s="7" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="I5" s="11"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>3</v>
       </c>
@@ -810,11 +827,14 @@
       <c r="F6" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G6" s="8" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="G6" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="I6" s="12" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>4</v>
       </c>
@@ -836,8 +856,9 @@
       <c r="G7" s="7" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="I7" s="11"/>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>5</v>
       </c>
@@ -859,6 +880,7 @@
       <c r="G8" s="7" t="s">
         <v>11</v>
       </c>
+      <c r="I8" s="11"/>
       <c r="J8" s="5" t="s">
         <v>26</v>
       </c>
@@ -866,7 +888,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>6</v>
       </c>
@@ -888,8 +910,9 @@
       <c r="G9" s="7" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="I9" s="11"/>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>7</v>
       </c>
@@ -914,13 +937,13 @@
       <c r="H10" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="I10" s="5" t="s">
+      <c r="I10" s="12" t="s">
         <v>56</v>
       </c>
       <c r="J10" s="5"/>
       <c r="K10" s="5"/>
     </row>
-    <row r="11" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>8</v>
       </c>
@@ -945,11 +968,11 @@
       <c r="H11" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="I11" s="5" t="s">
+      <c r="I11" s="12" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>9</v>
       </c>
@@ -974,11 +997,11 @@
       <c r="H12" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="I12" s="5" t="s">
+      <c r="I12" s="12" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>10</v>
       </c>
@@ -1000,8 +1023,9 @@
       <c r="G13" s="8" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="14" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="I13" s="11"/>
+    </row>
+    <row r="14" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>11</v>
       </c>
@@ -1026,7 +1050,7 @@
       <c r="H14" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="I14" s="5" t="s">
+      <c r="I14" s="12" t="s">
         <v>57</v>
       </c>
       <c r="J14" s="5" t="s">
@@ -1039,7 +1063,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>12</v>
       </c>
@@ -1058,11 +1082,17 @@
       <c r="F15" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G15" s="8" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="G15" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="H15" t="s">
+        <v>76</v>
+      </c>
+      <c r="I15" s="12" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>13</v>
       </c>
@@ -1084,8 +1114,9 @@
       <c r="G16" s="8" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="17" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="I16" s="11"/>
+    </row>
+    <row r="17" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>14</v>
       </c>
@@ -1107,11 +1138,11 @@
       <c r="G17" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="I17" s="5" t="s">
+      <c r="I17" s="12" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>15</v>
       </c>
@@ -1133,11 +1164,11 @@
       <c r="G18" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="I18" s="5" t="s">
+      <c r="I18" s="12" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>16</v>
       </c>
@@ -1159,11 +1190,11 @@
       <c r="G19" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="I19" s="5" t="s">
+      <c r="I19" s="12" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>17</v>
       </c>
@@ -1182,11 +1213,14 @@
       <c r="F20" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G20" s="8" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="G20" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="I20" s="12" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>18</v>
       </c>
@@ -1208,11 +1242,11 @@
       <c r="G21" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="I21" s="5" t="s">
+      <c r="I21" s="12" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>19</v>
       </c>
@@ -1234,8 +1268,9 @@
       <c r="G22" s="8" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I22" s="11"/>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>20</v>
       </c>
@@ -1257,8 +1292,9 @@
       <c r="G23" s="8" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="24" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="I23" s="11"/>
+    </row>
+    <row r="24" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>21</v>
       </c>
@@ -1280,8 +1316,9 @@
       <c r="G24" s="8" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I24" s="11"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>22</v>
       </c>
@@ -1303,71 +1340,90 @@
       <c r="G25" s="8" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I25" s="11"/>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C26" s="2"/>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I26" s="11"/>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C27" s="2"/>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I27" s="11"/>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C28" s="2"/>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I28" s="11"/>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C29" s="2"/>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I29" s="11"/>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C30" s="2"/>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I30" s="11"/>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C31" s="2"/>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I31" s="11"/>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C32" s="2"/>
-    </row>
-    <row r="33" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="I32" s="11"/>
+    </row>
+    <row r="33" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C33" s="2"/>
-    </row>
-    <row r="34" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="I33" s="11"/>
+    </row>
+    <row r="34" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C34" s="2"/>
-    </row>
-    <row r="35" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="I34" s="11"/>
+    </row>
+    <row r="35" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C35" s="2"/>
-    </row>
-    <row r="36" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="I35" s="11"/>
+    </row>
+    <row r="36" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C36" s="2"/>
-    </row>
-    <row r="37" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="I36" s="11"/>
+    </row>
+    <row r="37" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C37" s="2"/>
-    </row>
-    <row r="38" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="I37" s="11"/>
+    </row>
+    <row r="38" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C38" s="2"/>
-    </row>
-    <row r="39" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="I38" s="11"/>
+    </row>
+    <row r="39" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C39" s="2"/>
-    </row>
-    <row r="40" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="I39" s="11"/>
+    </row>
+    <row r="40" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C40" s="2"/>
-    </row>
-    <row r="41" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="I40" s="11"/>
+    </row>
+    <row r="41" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C41" s="2"/>
-    </row>
-    <row r="42" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="I41" s="11"/>
+    </row>
+    <row r="42" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C42" s="2"/>
-    </row>
-    <row r="43" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="I42" s="11"/>
+    </row>
+    <row r="43" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C43" s="2"/>
-    </row>
-    <row r="44" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="I43" s="11"/>
+    </row>
+    <row r="44" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C44" s="2"/>
     </row>
-    <row r="45" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C45" s="2"/>
     </row>
-    <row r="46" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C46" s="2"/>
     </row>
-    <row r="47" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C47" s="2"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new SW version - Aug 5th, 2026
</commit_message>
<xml_diff>
--- a/bug-tracker/UBA-bugs-tracker.xlsx
+++ b/bug-tracker/UBA-bugs-tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\DEV\UBA6-release\bug-tracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDC482B9-A172-4915-B771-24F2DCAA64DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A019E3FA-7E9E-4442-95A7-39CF379642DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{5B816FF3-3B79-4319-AB68-882518EDFCB6}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5B816FF3-3B79-4319-AB68-882518EDFCB6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="89">
   <si>
     <t>Num</t>
   </si>
@@ -207,16 +207,10 @@
     <t>checked in new version (28/7)</t>
   </si>
   <si>
-    <t>new feature in version (28/7)</t>
-  </si>
-  <si>
     <t>neet to consult with Tomer</t>
   </si>
   <si>
     <t>dc 4.8 v cuff off, then charge</t>
-  </si>
-  <si>
-    <t>inside test definition</t>
   </si>
   <si>
     <t>טעינה - DUAL</t>
@@ -284,13 +278,76 @@
   </si>
   <si>
     <t xml:space="preserve">כאשר נכנסים לרשימת התוכניות בנויות ולוחצים על אייקון  "צפיה" בתוכנית, לא ניתן ללחוץ על NEXT עד שלא מכניסים מספר סריאלי של המצבר. זה לא צריך להיות ככה. </t>
+  </si>
+  <si>
+    <t>database was overrided</t>
+  </si>
+  <si>
+    <t>new feature</t>
+  </si>
+  <si>
+    <t>3.08.2026</t>
+  </si>
+  <si>
+    <t>5.08.2026</t>
+  </si>
+  <si>
+    <t>Natasha, please show example of such fileName</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NEW FEATURE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> in version (28/7)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NEW FEATURE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, inside test definition</t>
+    </r>
+  </si>
+  <si>
+    <t>4.08.2026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -334,6 +391,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -361,7 +426,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -398,19 +463,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -764,19 +816,19 @@
         <v>6</v>
       </c>
       <c r="H3" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="J3" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="K3" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="L3" s="4" t="s">
         <v>69</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
@@ -801,6 +853,7 @@
       <c r="G4" s="7" t="s">
         <v>11</v>
       </c>
+      <c r="H4" s="5"/>
       <c r="J4" s="5" t="s">
         <v>26</v>
       </c>
@@ -830,6 +883,7 @@
       <c r="G5" s="7" t="s">
         <v>11</v>
       </c>
+      <c r="H5" s="5"/>
       <c r="I5" s="11"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
@@ -854,8 +908,9 @@
       <c r="G6" s="7" t="s">
         <v>11</v>
       </c>
+      <c r="H6" s="5"/>
       <c r="I6" s="12" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
@@ -880,6 +935,7 @@
       <c r="G7" s="7" t="s">
         <v>11</v>
       </c>
+      <c r="H7" s="5"/>
       <c r="I7" s="11"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
@@ -904,6 +960,7 @@
       <c r="G8" s="7" t="s">
         <v>11</v>
       </c>
+      <c r="H8" s="5"/>
       <c r="I8" s="11"/>
       <c r="J8" s="5" t="s">
         <v>26</v>
@@ -934,6 +991,7 @@
       <c r="G9" s="7" t="s">
         <v>11</v>
       </c>
+      <c r="H9" s="5"/>
       <c r="I9" s="11"/>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
@@ -1044,8 +1102,11 @@
       <c r="F13" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G13" s="8" t="s">
-        <v>18</v>
+      <c r="G13" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="I13" s="11"/>
     </row>
@@ -1068,23 +1129,23 @@
       <c r="F14" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G14" s="8" t="s">
+      <c r="G14" s="7" t="s">
         <v>11</v>
       </c>
       <c r="H14" s="5" t="s">
         <v>36</v>
       </c>
       <c r="I14" s="12" t="s">
-        <v>57</v>
+        <v>86</v>
       </c>
       <c r="J14" s="5" t="s">
         <v>26</v>
       </c>
       <c r="K14" s="9" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
@@ -1109,11 +1170,11 @@
       <c r="G15" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="H15" t="s">
-        <v>76</v>
+      <c r="H15" s="5" t="s">
+        <v>74</v>
       </c>
       <c r="I15" s="12" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -1138,7 +1199,10 @@
       <c r="G16" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="I16" s="11"/>
+      <c r="H16" s="5"/>
+      <c r="I16" s="11" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="17" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
@@ -1162,8 +1226,9 @@
       <c r="G17" s="8" t="s">
         <v>18</v>
       </c>
+      <c r="H17" s="5"/>
       <c r="I17" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
@@ -1188,8 +1253,9 @@
       <c r="G18" s="8" t="s">
         <v>18</v>
       </c>
+      <c r="H18" s="5"/>
       <c r="I18" s="12" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
@@ -1214,8 +1280,9 @@
       <c r="G19" s="8" t="s">
         <v>18</v>
       </c>
+      <c r="H19" s="5"/>
       <c r="I19" s="12" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
@@ -1240,8 +1307,11 @@
       <c r="G20" s="7" t="s">
         <v>11</v>
       </c>
+      <c r="H20" s="5" t="s">
+        <v>83</v>
+      </c>
       <c r="I20" s="12" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
@@ -1266,8 +1336,9 @@
       <c r="G21" s="8" t="s">
         <v>18</v>
       </c>
+      <c r="H21" s="5"/>
       <c r="I21" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
@@ -1292,6 +1363,7 @@
       <c r="G22" s="8" t="s">
         <v>18</v>
       </c>
+      <c r="H22" s="5"/>
       <c r="I22" s="11"/>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
@@ -1299,16 +1371,16 @@
         <v>20</v>
       </c>
       <c r="B23" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>55</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F23" s="5" t="s">
         <v>10</v>
@@ -1316,6 +1388,7 @@
       <c r="G23" s="8" t="s">
         <v>18</v>
       </c>
+      <c r="H23" s="5"/>
       <c r="I23" s="11"/>
     </row>
     <row r="24" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
@@ -1323,168 +1396,201 @@
         <v>21</v>
       </c>
       <c r="B24" t="s">
+        <v>62</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D24" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="C24" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>66</v>
-      </c>
       <c r="E24" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F24" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G24" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="I24" s="11"/>
+      <c r="G24" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="I24" s="11" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>22</v>
       </c>
       <c r="B25" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C25" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="H25" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="I25" s="11" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A26" s="1">
+        <v>23</v>
+      </c>
+      <c r="B26" t="s">
+        <v>77</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D26" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="D25" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="E25" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="F25" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="G25" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="I25" s="11"/>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A26" s="14">
-        <v>23</v>
-      </c>
-      <c r="B26" s="13" t="s">
+      <c r="E26" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G26" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="H26" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="I26" s="11" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A27" s="1">
+        <v>24</v>
+      </c>
+      <c r="B27" t="s">
         <v>79</v>
       </c>
-      <c r="C26" s="15" t="s">
+      <c r="C27" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="D26" s="16" t="s">
-        <v>76</v>
-      </c>
-      <c r="E26" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="F26" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="G26" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="H26" s="13"/>
-      <c r="I26" s="13"/>
-    </row>
-    <row r="27" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A27" s="14">
-        <v>24</v>
-      </c>
-      <c r="B27" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="C27" s="15" t="s">
-        <v>82</v>
-      </c>
-      <c r="D27" s="16" t="s">
-        <v>76</v>
-      </c>
-      <c r="E27" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="F27" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="G27" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="H27" s="13"/>
-      <c r="I27" s="13"/>
+      <c r="D27" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G27" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="H27" s="5" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C28" s="2"/>
+      <c r="H28" s="5"/>
       <c r="I28" s="11"/>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C29" s="2"/>
+      <c r="H29" s="5"/>
       <c r="I29" s="11"/>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C30" s="2"/>
+      <c r="H30" s="5"/>
       <c r="I30" s="11"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C31" s="2"/>
+      <c r="H31" s="5"/>
       <c r="I31" s="11"/>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C32" s="2"/>
+      <c r="H32" s="5"/>
       <c r="I32" s="11"/>
     </row>
     <row r="33" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C33" s="2"/>
+      <c r="H33" s="5"/>
       <c r="I33" s="11"/>
     </row>
     <row r="34" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C34" s="2"/>
+      <c r="H34" s="5"/>
       <c r="I34" s="11"/>
     </row>
     <row r="35" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C35" s="2"/>
+      <c r="H35" s="5"/>
       <c r="I35" s="11"/>
     </row>
     <row r="36" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C36" s="2"/>
+      <c r="H36" s="5"/>
       <c r="I36" s="11"/>
     </row>
     <row r="37" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C37" s="2"/>
+      <c r="H37" s="5"/>
       <c r="I37" s="11"/>
     </row>
     <row r="38" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C38" s="2"/>
+      <c r="H38" s="5"/>
       <c r="I38" s="11"/>
     </row>
     <row r="39" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C39" s="2"/>
+      <c r="H39" s="5"/>
       <c r="I39" s="11"/>
     </row>
     <row r="40" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C40" s="2"/>
+      <c r="H40" s="5"/>
       <c r="I40" s="11"/>
     </row>
     <row r="41" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C41" s="2"/>
+      <c r="H41" s="5"/>
       <c r="I41" s="11"/>
     </row>
     <row r="42" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C42" s="2"/>
+      <c r="H42" s="5"/>
       <c r="I42" s="11"/>
     </row>
     <row r="43" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C43" s="2"/>
+      <c r="H43" s="5"/>
       <c r="I43" s="11"/>
     </row>
     <row r="44" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C44" s="2"/>
+      <c r="H44" s="5"/>
     </row>
     <row r="45" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C45" s="2"/>
+      <c r="H45" s="5"/>
     </row>
     <row r="46" spans="3:9" x14ac:dyDescent="0.3">
       <c r="C46" s="2"/>

</xml_diff>